<commit_message>
fix structure both system
</commit_message>
<xml_diff>
--- a/خصومات الاسنان - Copy.xlsx
+++ b/خصومات الاسنان - Copy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Omar\waad_temp_website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13F45782-62E4-4B66-A8D4-23C84DA31A9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA5161DC-8539-4404-98CD-A4F68702FB95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="الاسنان " sheetId="3" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'الاسنان '!$D$204:$D$227</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'الاسنان '!$B$1:$H$78</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -7652,7 +7652,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="307">
+  <cellXfs count="306">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
@@ -8523,9 +8523,6 @@
       <alignment horizontal="center" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9060,6 +9057,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EFF41BA-9577-4F85-9F07-37B4DCE13C1E}">
+  <sheetPr filterMode="1"/>
   <dimension ref="B1:K1094"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
@@ -9095,7 +9093,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="2" spans="2:8" ht="18" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:8" ht="18" hidden="1" x14ac:dyDescent="0.35">
       <c r="B2" s="15" t="s">
         <v>401</v>
       </c>
@@ -9118,7 +9116,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="3" spans="2:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:8" ht="21" hidden="1" x14ac:dyDescent="0.4">
       <c r="B3" s="21" t="s">
         <v>404</v>
       </c>
@@ -9141,7 +9139,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="4" spans="2:8" ht="18" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:8" ht="18" hidden="1" x14ac:dyDescent="0.35">
       <c r="B4" s="21" t="s">
         <v>407</v>
       </c>
@@ -9164,7 +9162,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="5" spans="2:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:8" ht="21" hidden="1" x14ac:dyDescent="0.4">
       <c r="B5" s="42" t="s">
         <v>409</v>
       </c>
@@ -9187,7 +9185,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:8" ht="21" hidden="1" x14ac:dyDescent="0.4">
       <c r="B6" s="21" t="s">
         <v>411</v>
       </c>
@@ -9210,7 +9208,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="7" spans="2:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:8" ht="21" hidden="1" x14ac:dyDescent="0.4">
       <c r="B7" s="104" t="s">
         <v>413</v>
       </c>
@@ -9233,7 +9231,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="8" spans="2:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:8" ht="21" hidden="1" x14ac:dyDescent="0.4">
       <c r="B8" s="41" t="s">
         <v>415</v>
       </c>
@@ -9256,7 +9254,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="9" spans="2:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:8" ht="21" hidden="1" x14ac:dyDescent="0.4">
       <c r="B9" s="7" t="s">
         <v>418</v>
       </c>
@@ -9279,7 +9277,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="10" spans="2:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:8" ht="21" hidden="1" x14ac:dyDescent="0.4">
       <c r="B10" s="21" t="s">
         <v>420</v>
       </c>
@@ -9302,7 +9300,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="11" spans="2:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:8" ht="21" hidden="1" x14ac:dyDescent="0.4">
       <c r="B11" s="5" t="s">
         <v>423</v>
       </c>
@@ -9325,7 +9323,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="12" spans="2:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:8" ht="21" hidden="1" x14ac:dyDescent="0.4">
       <c r="B12" s="21" t="s">
         <v>425</v>
       </c>
@@ -9348,7 +9346,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="13" spans="2:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:8" ht="21" hidden="1" x14ac:dyDescent="0.4">
       <c r="B13" s="27" t="s">
         <v>427</v>
       </c>
@@ -9371,7 +9369,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="14" spans="2:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:8" ht="21" hidden="1" x14ac:dyDescent="0.4">
       <c r="B14" s="14" t="s">
         <v>430</v>
       </c>
@@ -9394,7 +9392,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="15" spans="2:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:8" ht="21" hidden="1" x14ac:dyDescent="0.4">
       <c r="B15" s="14" t="s">
         <v>431</v>
       </c>
@@ -9417,7 +9415,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="16" spans="2:8" ht="21" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:8" ht="21" hidden="1" x14ac:dyDescent="0.35">
       <c r="B16" s="27" t="s">
         <v>433</v>
       </c>
@@ -9440,7 +9438,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="17" spans="2:8" ht="21" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:8" ht="21" hidden="1" x14ac:dyDescent="0.35">
       <c r="B17" s="14" t="s">
         <v>435</v>
       </c>
@@ -9463,7 +9461,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="18" spans="2:8" ht="21" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:8" ht="21" hidden="1" x14ac:dyDescent="0.35">
       <c r="B18" s="27" t="s">
         <v>437</v>
       </c>
@@ -9486,7 +9484,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="19" spans="2:8" ht="18" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:8" ht="18" hidden="1" x14ac:dyDescent="0.35">
       <c r="B19" s="245" t="s">
         <v>438</v>
       </c>
@@ -9509,7 +9507,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="20" spans="2:8" ht="18" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:8" ht="18" hidden="1" x14ac:dyDescent="0.35">
       <c r="B20" s="246" t="s">
         <v>440</v>
       </c>
@@ -9532,7 +9530,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="21" spans="2:8" ht="18.600000000000001" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:8" ht="18.600000000000001" hidden="1" x14ac:dyDescent="0.35">
       <c r="B21" s="77" t="s">
         <v>442</v>
       </c>
@@ -9555,7 +9553,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="22" spans="2:8" ht="18" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:8" ht="18" hidden="1" x14ac:dyDescent="0.3">
       <c r="B22" s="33" t="s">
         <v>444</v>
       </c>
@@ -9578,7 +9576,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="23" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B23" s="33" t="s">
         <v>447</v>
       </c>
@@ -9601,7 +9599,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="24" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B24" s="33" t="s">
         <v>450</v>
       </c>
@@ -9622,7 +9620,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="25" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B25" s="33" t="s">
         <v>453</v>
       </c>
@@ -9643,7 +9641,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="26" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B26" s="33" t="s">
         <v>456</v>
       </c>
@@ -9666,7 +9664,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="27" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B27" s="33" t="s">
         <v>460</v>
       </c>
@@ -9687,7 +9685,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="28" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B28" s="33" t="s">
         <v>411</v>
       </c>
@@ -9710,7 +9708,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="29" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B29" s="38" t="s">
         <v>465</v>
       </c>
@@ -9731,7 +9729,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="30" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B30" s="33" t="s">
         <v>437</v>
       </c>
@@ -9752,7 +9750,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="31" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B31" s="33" t="s">
         <v>273</v>
       </c>
@@ -9773,7 +9771,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="32" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B32" s="33" t="s">
         <v>273</v>
       </c>
@@ -9794,7 +9792,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="33" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B33" s="33" t="s">
         <v>472</v>
       </c>
@@ -9815,7 +9813,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="34" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B34" s="33" t="s">
         <v>475</v>
       </c>
@@ -9836,7 +9834,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="35" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B35" s="33" t="s">
         <v>478</v>
       </c>
@@ -9857,7 +9855,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="36" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B36" s="33" t="s">
         <v>433</v>
       </c>
@@ -9880,7 +9878,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="37" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B37" s="33" t="s">
         <v>483</v>
       </c>
@@ -9922,7 +9920,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="39" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B39" s="204" t="s">
         <v>490</v>
       </c>
@@ -9945,7 +9943,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="40" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B40" s="33" t="s">
         <v>478</v>
       </c>
@@ -9966,7 +9964,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="41" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B41" s="33" t="s">
         <v>494</v>
       </c>
@@ -9987,7 +9985,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="42" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B42" s="33" t="s">
         <v>496</v>
       </c>
@@ -10008,7 +10006,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="43" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B43" s="33" t="s">
         <v>496</v>
       </c>
@@ -10029,7 +10027,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="44" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B44" s="33" t="s">
         <v>500</v>
       </c>
@@ -10050,7 +10048,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="45" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B45" s="33" t="s">
         <v>504</v>
       </c>
@@ -10071,7 +10069,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="46" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B46" s="33" t="s">
         <v>494</v>
       </c>
@@ -10092,7 +10090,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="47" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B47" s="33" t="s">
         <v>508</v>
       </c>
@@ -10113,7 +10111,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="48" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B48" s="33" t="s">
         <v>511</v>
       </c>
@@ -10176,7 +10174,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="51" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B51" s="33" t="s">
         <v>516</v>
       </c>
@@ -10197,7 +10195,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="52" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B52" s="33" t="s">
         <v>519</v>
       </c>
@@ -10218,7 +10216,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="53" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B53" s="33" t="s">
         <v>522</v>
       </c>
@@ -10239,7 +10237,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="54" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B54" s="38" t="s">
         <v>525</v>
       </c>
@@ -10260,7 +10258,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="55" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B55" s="33" t="s">
         <v>527</v>
       </c>
@@ -10281,7 +10279,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="56" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B56" s="37" t="s">
         <v>530</v>
       </c>
@@ -10302,7 +10300,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="57" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B57" s="33" t="s">
         <v>532</v>
       </c>
@@ -10323,7 +10321,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="58" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B58" s="33" t="s">
         <v>534</v>
       </c>
@@ -10344,7 +10342,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="59" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B59" s="33" t="s">
         <v>535</v>
       </c>
@@ -10386,7 +10384,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="61" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B61" s="33" t="s">
         <v>537</v>
       </c>
@@ -10407,7 +10405,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="62" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B62" s="37" t="s">
         <v>530</v>
       </c>
@@ -10428,7 +10426,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="63" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B63" s="33" t="s">
         <v>539</v>
       </c>
@@ -10449,7 +10447,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="64" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B64" s="33" t="s">
         <v>540</v>
       </c>
@@ -10470,7 +10468,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="65" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B65" s="33" t="s">
         <v>541</v>
       </c>
@@ -10491,7 +10489,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="66" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B66" s="33" t="s">
         <v>543</v>
       </c>
@@ -10512,7 +10510,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="67" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B67" s="33" t="s">
         <v>545</v>
       </c>
@@ -10533,7 +10531,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="68" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B68" s="33" t="s">
         <v>546</v>
       </c>
@@ -10554,7 +10552,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="69" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B69" s="33" t="s">
         <v>293</v>
       </c>
@@ -10575,7 +10573,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="70" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B70" s="33" t="s">
         <v>550</v>
       </c>
@@ -10619,7 +10617,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="72" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B72" s="33" t="s">
         <v>546</v>
       </c>
@@ -10640,7 +10638,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="73" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B73" s="33" t="s">
         <v>556</v>
       </c>
@@ -10661,7 +10659,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="74" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B74" s="33" t="s">
         <v>558</v>
       </c>
@@ -10682,7 +10680,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="75" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B75" s="33" t="s">
         <v>273</v>
       </c>
@@ -10703,7 +10701,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="76" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B76" s="33" t="s">
         <v>563</v>
       </c>
@@ -10724,7 +10722,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="77" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B77" s="33" t="s">
         <v>263</v>
       </c>
@@ -10745,7 +10743,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="78" spans="2:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:8" ht="17.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="B78" s="33"/>
       <c r="C78" s="33" t="s">
         <v>56</v>
@@ -30344,7 +30342,7 @@
       <c r="G1091" s="253" t="s">
         <v>529</v>
       </c>
-      <c r="H1091" s="306" t="s">
+      <c r="H1091" s="219" t="s">
         <v>2333</v>
       </c>
     </row>
@@ -30367,7 +30365,7 @@
       <c r="G1092" s="253" t="s">
         <v>626</v>
       </c>
-      <c r="H1092" s="306" t="s">
+      <c r="H1092" s="219" t="s">
         <v>2333</v>
       </c>
     </row>
@@ -30390,7 +30388,7 @@
       <c r="G1093" s="253" t="s">
         <v>626</v>
       </c>
-      <c r="H1093" s="306" t="s">
+      <c r="H1093" s="219" t="s">
         <v>2333</v>
       </c>
     </row>
@@ -30413,12 +30411,18 @@
       <c r="G1094" s="253" t="s">
         <v>626</v>
       </c>
-      <c r="H1094" s="306" t="s">
+      <c r="H1094" s="219" t="s">
         <v>2333</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="D204:D227" xr:uid="{1EFF41BA-9577-4F85-9F07-37B4DCE13C1E}"/>
+  <autoFilter ref="B1:H78" xr:uid="{1EFF41BA-9577-4F85-9F07-37B4DCE13C1E}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="نجلاء فتحي مفتاح عمر"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>